<commit_message>
Add confidence interval problem summary sheet to Excel file
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ara64wtPcoNHRrRRFpeXXp
</commit_message>
<xml_diff>
--- a/24rd006_飯島悠矢.xlsx
+++ b/24rd006_飯島悠矢.xlsx
@@ -7,12 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="t分布" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="tanh" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="tanh-1" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="二項分布累積" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="正規分布累積" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="正規分布逆関数" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="問題_信頼区間" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="t分布" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="tanh" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="tanh-1" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="二項分布累積" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="正規分布累積" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="正規分布逆関数" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,16 +31,54 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DEEAF1"/>
+        <bgColor rgb="00DEEAF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +86,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,6 +490,289 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B1:E31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>統計学Ⅰ 第10回 問題解答　─　相関係数の区間推定</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="8" customHeight="1"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>【問題】</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>サンプル数 N=20 のデータから r=0.3 の相関係数が得られた。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>① この時の 95% 信頼区間を求めよ。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>② 同じデータの 99% 信頼区間を求めよ。（標準正規分布の上側確率 0.5% となる x = 2.567）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="8" customHeight="1"/>
+    <row r="8" ht="22" customHeight="1">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>【解法】フィッシャーのZ変換による区間推定</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>▶ Step 1：標本相関係数 r を Z 変換する</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Z = tanh⁻¹(r) = ATANH(0.3)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Z ≈ 0.3095</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>▶ Step 2：Z の標準誤差を求める</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>SE = 1 / √(N−3) = 1 / √17</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>SE ≈ 0.2425</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>▶ Step 3：Z の信頼区間を求め、tanh で ρ の信頼区間に変換する</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="8" customHeight="1"/>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>【計算結果】</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="6" t="inlineStr"/>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>z* の値</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Z の下限 / 上限</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>ρ の信頼区間</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>95% 信頼区間</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>z* = 1.96</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Z: −0.1658 ～ 0.7848</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>−0.165 &lt; ρ &lt; 0.656</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>99% 信頼区間</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>z* = 2.567</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Z: −0.3130 ～ 0.9320</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>−0.306 &lt; ρ &lt; 0.730</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="8" customHeight="1"/>
+    <row r="20" ht="22" customHeight="1">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>【計算過程の詳細】</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>95% 信頼区間の計算</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Z − 1.96/√17  =  0.3095 − 0.4753  =  −0.1658  →  tanh(−0.1658) ≈ −0.165</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Z + 1.96/√17  =  0.3095 + 0.4753  =   0.7848  →  tanh( 0.7848) ≈  0.656</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="B24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>99% 信頼区間の計算</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Z − 2.567/√17  =  0.3095 − 0.6225  =  −0.3130  →  tanh(−0.3130) ≈ −0.306</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Z + 2.567/√17  =  0.3095 + 0.6225  =   0.9320  →  tanh( 0.9320) ≈  0.730</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="8" customHeight="1"/>
+    <row r="29" ht="22" customHeight="1">
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>【考察】</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>信頼水準を 95% → 99% に上げると、信頼区間が広くなる（より確実に母数を含む分、範囲が拡大する）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>r=0.3 は N=20 では有意ではない可能性があり、信頼区間がゼロをまたいでいることからも確認できる。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="25">
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B29:E29"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -967,7 +1322,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1992,7 +2347,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4007,7 +4362,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4322,7 +4677,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4930,7 +5285,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Simplify problem summary sheet to plain black and white format
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ara64wtPcoNHRrRRFpeXXp
</commit_message>
<xml_diff>
--- a/24rd006_飯島悠矢.xlsx
+++ b/24rd006_飯島悠矢.xlsx
@@ -78,7 +78,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -92,11 +92,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -124,6 +152,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -490,279 +524,132 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E31"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="B1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>統計学Ⅰ 第10回 問題解答　─　相関係数の区間推定</t>
+          <t>統計学Ⅰ 第10回　問題解答</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="8" customHeight="1"/>
-    <row r="3" ht="22" customHeight="1">
-      <c r="B3" s="2" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>【問題】</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>サンプル数 N=20 のデータから r=0.3 の相関係数が得られた。</t>
+          <t>N=20、r=0.3 の相関係数が得られた。</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>① この時の 95% 信頼区間を求めよ。</t>
+          <t>① 95% 信頼区間を求めよ。</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="B6" s="3" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>② 同じデータの 99% 信頼区間を求めよ。（標準正規分布の上側確率 0.5% となる x = 2.567）</t>
+          <t>② 99% 信頼区間を求めよ。（z*=2.567）</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="8" customHeight="1"/>
-    <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>【解法】フィッシャーのZ変換による区間推定</t>
+          <t>【解法】フィッシャーのZ変換</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>▶ Step 1：標本相関係数 r を Z 変換する</t>
+          <t>Z = ATANH(0.3) ≈ 0.3095</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Z = tanh⁻¹(r) = ATANH(0.3)</t>
+          <t>SE = 1/√(N-3) = 1/√17 ≈ 0.2425</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>Z ≈ 0.3095</t>
+          <t>信頼区間: tanh(Z ± z*/√(N-3))</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>▶ Step 2：Z の標準誤差を求める</t>
+          <t>【答え】</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>SE = 1 / √(N−3) = 1 / √17</t>
+          <t>95%: -0.165 &lt; ρ &lt; 0.656</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>SE ≈ 0.2425</t>
+          <t>99%: -0.306 &lt; ρ &lt; 0.730</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>▶ Step 3：Z の信頼区間を求め、tanh で ρ の信頼区間に変換する</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="8" customHeight="1"/>
-    <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>【計算結果】</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="6" t="inlineStr"/>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>z* の値</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>Z の下限 / 上限</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>ρ の信頼区間</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>95% 信頼区間</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>z* = 1.96</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Z: −0.1658 ～ 0.7848</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>−0.165 &lt; ρ &lt; 0.656</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>99% 信頼区間</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>z* = 2.567</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Z: −0.3130 ～ 0.9320</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>−0.306 &lt; ρ &lt; 0.730</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="8" customHeight="1"/>
-    <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>【計算過程の詳細】</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>95% 信頼区間の計算</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Z − 1.96/√17  =  0.3095 − 0.4753  =  −0.1658  →  tanh(−0.1658) ≈ −0.165</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Z + 1.96/√17  =  0.3095 + 0.4753  =   0.7848  →  tanh( 0.7848) ≈  0.656</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="B24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>99% 信頼区間の計算</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Z − 2.567/√17  =  0.3095 − 0.6225  =  −0.3130  →  tanh(−0.3130) ≈ −0.306</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Z + 2.567/√17  =  0.3095 + 0.6225  =   0.9320  →  tanh( 0.9320) ≈  0.730</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="8" customHeight="1"/>
-    <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>【考察】</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="B30" s="3" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>信頼水準を 95% → 99% に上げると、信頼区間が広くなる（より確実に母数を含む分、範囲が拡大する）。</t>
+          <t>信頼水準を上げると信頼区間は広くなる。</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="24" customHeight="1">
-      <c r="B31" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>r=0.3 は N=20 では有意ではない可能性があり、信頼区間がゼロをまたいでいることからも確認できる。</t>
+          <t>信頼区間がゼロをまたぐため、r=0.3 は有意でない可能性がある。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B20:E20"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B29:E29"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update problem sheet to show values in PDF-style format
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ara64wtPcoNHRrRRFpeXXp
</commit_message>
<xml_diff>
--- a/24rd006_飯島悠矢.xlsx
+++ b/24rd006_飯島悠矢.xlsx
@@ -124,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -158,6 +158,11 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -524,128 +529,150 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>統計学Ⅰ 第10回　問題解答</t>
+          <t>統計学Ⅰ 第10回　問題</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr"/>
+      <c r="A2" s="13" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>【問題】</t>
+          <t>N = 20,  r = 0.3</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>N=20、r=0.3 の相関係数が得られた。</t>
+          <t>① 95% 信頼区間</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>① 95% 信頼区間を求めよ。</t>
+          <t>Z = ATANH(0.3)</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>② 99% 信頼区間を求めよ。（z*=2.567）</t>
+          <t>=</t>
         </is>
       </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>0.3095</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr"/>
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>SE = 1/√(20−3)</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>0.2425</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>【解法】フィッシャーのZ変換</t>
+          <t>Z ± 1.96 × SE</t>
         </is>
       </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>−0.1658  ～  0.7848</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>Z = ATANH(0.3) ≈ 0.3095</t>
+          <t>tanh(下限), tanh(上限)</t>
         </is>
       </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>−0.165  &lt;  ρ  &lt;  0.656</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>SE = 1/√(N-3) = 1/√17 ≈ 0.2425</t>
+          <t>② 99% 信頼区間  (z* = 2.567)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>信頼区間: tanh(Z ± z*/√(N-3))</t>
+          <t>Z ± 2.567 × SE</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="11" t="inlineStr"/>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>−0.3130  ～  0.9320</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>【答え】</t>
+          <t>tanh(下限), tanh(上限)</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>95%: -0.165 &lt; ρ &lt; 0.656</t>
+          <t>→</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>99%: -0.306 &lt; ρ &lt; 0.730</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>【考察】</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>信頼水準を上げると信頼区間は広くなる。</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>信頼区間がゼロをまたぐため、r=0.3 は有意でない可能性がある。</t>
+          <t>−0.306  &lt;  ρ  &lt;  0.730</t>
         </is>
       </c>
     </row>

</xml_diff>